<commit_message>
Format visitor log date/time column as dd/mm/yyyy hh:mm
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013FUkLGmYvKevpCsh9ZXdui
</commit_message>
<xml_diff>
--- a/resources/سجل_الزائرات_للمدرسة.xlsx
+++ b/resources/سجل_الزائرات_للمدرسة.xlsx
@@ -20,7 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy hh:mm"/>
+  </numFmts>
   <fonts count="7">
     <font>
       <name val="Calibri"/>
@@ -88,7 +90,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -124,11 +126,55 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -167,6 +213,14 @@
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
@@ -560,17 +614,17 @@
           <t>اسم المدرسة:</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
+      <c r="B2" s="14" t="n"/>
       <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="14" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>العام الدراسي:</t>
         </is>
       </c>
       <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
+      <c r="H2" s="14" t="n"/>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="36" customHeight="1">
@@ -619,7 +673,7 @@
       <c r="A5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="7" t="n"/>
+      <c r="B5" s="16" t="n"/>
       <c r="C5" s="8" t="n"/>
       <c r="D5" s="9" t="n"/>
       <c r="E5" s="8" t="n"/>
@@ -631,7 +685,7 @@
       <c r="A6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="11" t="n"/>
+      <c r="B6" s="17" t="n"/>
       <c r="C6" s="12" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="12" t="n"/>
@@ -643,7 +697,7 @@
       <c r="A7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="7" t="n"/>
+      <c r="B7" s="16" t="n"/>
       <c r="C7" s="8" t="n"/>
       <c r="D7" s="9" t="n"/>
       <c r="E7" s="8" t="n"/>
@@ -655,7 +709,7 @@
       <c r="A8" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="11" t="n"/>
+      <c r="B8" s="17" t="n"/>
       <c r="C8" s="12" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="12" t="n"/>
@@ -667,7 +721,7 @@
       <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="7" t="n"/>
+      <c r="B9" s="16" t="n"/>
       <c r="C9" s="8" t="n"/>
       <c r="D9" s="9" t="n"/>
       <c r="E9" s="8" t="n"/>
@@ -679,7 +733,7 @@
       <c r="A10" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="11" t="n"/>
+      <c r="B10" s="17" t="n"/>
       <c r="C10" s="12" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="12" t="n"/>
@@ -691,7 +745,7 @@
       <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="7" t="n"/>
+      <c r="B11" s="16" t="n"/>
       <c r="C11" s="8" t="n"/>
       <c r="D11" s="9" t="n"/>
       <c r="E11" s="8" t="n"/>
@@ -703,7 +757,7 @@
       <c r="A12" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="11" t="n"/>
+      <c r="B12" s="17" t="n"/>
       <c r="C12" s="12" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="12" t="n"/>
@@ -715,7 +769,7 @@
       <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="7" t="n"/>
+      <c r="B13" s="16" t="n"/>
       <c r="C13" s="8" t="n"/>
       <c r="D13" s="9" t="n"/>
       <c r="E13" s="8" t="n"/>
@@ -727,7 +781,7 @@
       <c r="A14" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="11" t="n"/>
+      <c r="B14" s="17" t="n"/>
       <c r="C14" s="12" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="12" t="n"/>
@@ -739,7 +793,7 @@
       <c r="A15" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="7" t="n"/>
+      <c r="B15" s="16" t="n"/>
       <c r="C15" s="8" t="n"/>
       <c r="D15" s="9" t="n"/>
       <c r="E15" s="8" t="n"/>
@@ -751,7 +805,7 @@
       <c r="A16" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="11" t="n"/>
+      <c r="B16" s="17" t="n"/>
       <c r="C16" s="12" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="12" t="n"/>
@@ -763,7 +817,7 @@
       <c r="A17" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="7" t="n"/>
+      <c r="B17" s="16" t="n"/>
       <c r="C17" s="8" t="n"/>
       <c r="D17" s="9" t="n"/>
       <c r="E17" s="8" t="n"/>
@@ -775,7 +829,7 @@
       <c r="A18" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="11" t="n"/>
+      <c r="B18" s="17" t="n"/>
       <c r="C18" s="12" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="12" t="n"/>
@@ -787,7 +841,7 @@
       <c r="A19" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="7" t="n"/>
+      <c r="B19" s="16" t="n"/>
       <c r="C19" s="8" t="n"/>
       <c r="D19" s="9" t="n"/>
       <c r="E19" s="8" t="n"/>
@@ -799,7 +853,7 @@
       <c r="A20" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="11" t="n"/>
+      <c r="B20" s="17" t="n"/>
       <c r="C20" s="12" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="12" t="n"/>
@@ -811,7 +865,7 @@
       <c r="A21" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="7" t="n"/>
+      <c r="B21" s="16" t="n"/>
       <c r="C21" s="8" t="n"/>
       <c r="D21" s="9" t="n"/>
       <c r="E21" s="8" t="n"/>
@@ -823,7 +877,7 @@
       <c r="A22" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="11" t="n"/>
+      <c r="B22" s="17" t="n"/>
       <c r="C22" s="12" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="12" t="n"/>
@@ -835,7 +889,7 @@
       <c r="A23" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="7" t="n"/>
+      <c r="B23" s="16" t="n"/>
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="8" t="n"/>
@@ -847,7 +901,7 @@
       <c r="A24" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="11" t="n"/>
+      <c r="B24" s="17" t="n"/>
       <c r="C24" s="12" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="12" t="n"/>
@@ -859,7 +913,7 @@
       <c r="A25" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="7" t="n"/>
+      <c r="B25" s="16" t="n"/>
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="8" t="n"/>
@@ -871,7 +925,7 @@
       <c r="A26" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="11" t="n"/>
+      <c r="B26" s="17" t="n"/>
       <c r="C26" s="12" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="12" t="n"/>
@@ -883,7 +937,7 @@
       <c r="A27" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="7" t="n"/>
+      <c r="B27" s="16" t="n"/>
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="8" t="n"/>
@@ -895,7 +949,7 @@
       <c r="A28" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="11" t="n"/>
+      <c r="B28" s="17" t="n"/>
       <c r="C28" s="12" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="12" t="n"/>
@@ -907,7 +961,7 @@
       <c r="A29" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="7" t="n"/>
+      <c r="B29" s="16" t="n"/>
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="8" t="n"/>
@@ -919,7 +973,7 @@
       <c r="A30" s="10" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="11" t="n"/>
+      <c r="B30" s="17" t="n"/>
       <c r="C30" s="12" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="12" t="n"/>
@@ -931,7 +985,7 @@
       <c r="A31" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="7" t="n"/>
+      <c r="B31" s="16" t="n"/>
       <c r="C31" s="8" t="n"/>
       <c r="D31" s="9" t="n"/>
       <c r="E31" s="8" t="n"/>
@@ -943,7 +997,7 @@
       <c r="A32" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="11" t="n"/>
+      <c r="B32" s="17" t="n"/>
       <c r="C32" s="12" t="n"/>
       <c r="D32" s="13" t="n"/>
       <c r="E32" s="12" t="n"/>
@@ -955,7 +1009,7 @@
       <c r="A33" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="7" t="n"/>
+      <c r="B33" s="16" t="n"/>
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="9" t="n"/>
       <c r="E33" s="8" t="n"/>
@@ -967,7 +1021,7 @@
       <c r="A34" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="11" t="n"/>
+      <c r="B34" s="17" t="n"/>
       <c r="C34" s="12" t="n"/>
       <c r="D34" s="13" t="n"/>
       <c r="E34" s="12" t="n"/>
@@ -979,7 +1033,7 @@
       <c r="A35" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="7" t="n"/>
+      <c r="B35" s="16" t="n"/>
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="9" t="n"/>
       <c r="E35" s="8" t="n"/>
@@ -991,7 +1045,7 @@
       <c r="A36" s="10" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="11" t="n"/>
+      <c r="B36" s="17" t="n"/>
       <c r="C36" s="12" t="n"/>
       <c r="D36" s="13" t="n"/>
       <c r="E36" s="12" t="n"/>
@@ -1003,7 +1057,7 @@
       <c r="A37" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="7" t="n"/>
+      <c r="B37" s="16" t="n"/>
       <c r="C37" s="8" t="n"/>
       <c r="D37" s="9" t="n"/>
       <c r="E37" s="8" t="n"/>
@@ -1015,7 +1069,7 @@
       <c r="A38" s="10" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="11" t="n"/>
+      <c r="B38" s="17" t="n"/>
       <c r="C38" s="12" t="n"/>
       <c r="D38" s="13" t="n"/>
       <c r="E38" s="12" t="n"/>
@@ -1027,7 +1081,7 @@
       <c r="A39" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="7" t="n"/>
+      <c r="B39" s="16" t="n"/>
       <c r="C39" s="8" t="n"/>
       <c r="D39" s="9" t="n"/>
       <c r="E39" s="8" t="n"/>
@@ -1039,7 +1093,7 @@
       <c r="A40" s="10" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="11" t="n"/>
+      <c r="B40" s="17" t="n"/>
       <c r="C40" s="12" t="n"/>
       <c r="D40" s="13" t="n"/>
       <c r="E40" s="12" t="n"/>
@@ -1051,7 +1105,7 @@
       <c r="A41" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="7" t="n"/>
+      <c r="B41" s="16" t="n"/>
       <c r="C41" s="8" t="n"/>
       <c r="D41" s="9" t="n"/>
       <c r="E41" s="8" t="n"/>
@@ -1063,7 +1117,7 @@
       <c r="A42" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="11" t="n"/>
+      <c r="B42" s="17" t="n"/>
       <c r="C42" s="12" t="n"/>
       <c r="D42" s="13" t="n"/>
       <c r="E42" s="12" t="n"/>
@@ -1075,7 +1129,7 @@
       <c r="A43" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="7" t="n"/>
+      <c r="B43" s="16" t="n"/>
       <c r="C43" s="8" t="n"/>
       <c r="D43" s="9" t="n"/>
       <c r="E43" s="8" t="n"/>
@@ -1087,7 +1141,7 @@
       <c r="A44" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="11" t="n"/>
+      <c r="B44" s="17" t="n"/>
       <c r="C44" s="12" t="n"/>
       <c r="D44" s="13" t="n"/>
       <c r="E44" s="12" t="n"/>
@@ -1099,7 +1153,7 @@
       <c r="A45" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="B45" s="7" t="n"/>
+      <c r="B45" s="16" t="n"/>
       <c r="C45" s="8" t="n"/>
       <c r="D45" s="9" t="n"/>
       <c r="E45" s="8" t="n"/>
@@ -1111,7 +1165,7 @@
       <c r="A46" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="11" t="n"/>
+      <c r="B46" s="17" t="n"/>
       <c r="C46" s="12" t="n"/>
       <c r="D46" s="13" t="n"/>
       <c r="E46" s="12" t="n"/>
@@ -1123,7 +1177,7 @@
       <c r="A47" s="6" t="n">
         <v>43</v>
       </c>
-      <c r="B47" s="7" t="n"/>
+      <c r="B47" s="16" t="n"/>
       <c r="C47" s="8" t="n"/>
       <c r="D47" s="9" t="n"/>
       <c r="E47" s="8" t="n"/>
@@ -1135,7 +1189,7 @@
       <c r="A48" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="11" t="n"/>
+      <c r="B48" s="17" t="n"/>
       <c r="C48" s="12" t="n"/>
       <c r="D48" s="13" t="n"/>
       <c r="E48" s="12" t="n"/>
@@ -1147,7 +1201,7 @@
       <c r="A49" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="B49" s="7" t="n"/>
+      <c r="B49" s="16" t="n"/>
       <c r="C49" s="8" t="n"/>
       <c r="D49" s="9" t="n"/>
       <c r="E49" s="8" t="n"/>
@@ -1159,7 +1213,7 @@
       <c r="A50" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="B50" s="11" t="n"/>
+      <c r="B50" s="17" t="n"/>
       <c r="C50" s="12" t="n"/>
       <c r="D50" s="13" t="n"/>
       <c r="E50" s="12" t="n"/>
@@ -1171,7 +1225,7 @@
       <c r="A51" s="6" t="n">
         <v>47</v>
       </c>
-      <c r="B51" s="7" t="n"/>
+      <c r="B51" s="16" t="n"/>
       <c r="C51" s="8" t="n"/>
       <c r="D51" s="9" t="n"/>
       <c r="E51" s="8" t="n"/>
@@ -1183,7 +1237,7 @@
       <c r="A52" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="B52" s="11" t="n"/>
+      <c r="B52" s="17" t="n"/>
       <c r="C52" s="12" t="n"/>
       <c r="D52" s="13" t="n"/>
       <c r="E52" s="12" t="n"/>
@@ -1195,7 +1249,7 @@
       <c r="A53" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="B53" s="7" t="n"/>
+      <c r="B53" s="16" t="n"/>
       <c r="C53" s="8" t="n"/>
       <c r="D53" s="9" t="n"/>
       <c r="E53" s="8" t="n"/>
@@ -1207,7 +1261,7 @@
       <c r="A54" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="B54" s="11" t="n"/>
+      <c r="B54" s="17" t="n"/>
       <c r="C54" s="12" t="n"/>
       <c r="D54" s="13" t="n"/>
       <c r="E54" s="12" t="n"/>
@@ -1219,7 +1273,7 @@
       <c r="A55" s="6" t="n">
         <v>51</v>
       </c>
-      <c r="B55" s="7" t="n"/>
+      <c r="B55" s="16" t="n"/>
       <c r="C55" s="8" t="n"/>
       <c r="D55" s="9" t="n"/>
       <c r="E55" s="8" t="n"/>
@@ -1231,7 +1285,7 @@
       <c r="A56" s="10" t="n">
         <v>52</v>
       </c>
-      <c r="B56" s="11" t="n"/>
+      <c r="B56" s="17" t="n"/>
       <c r="C56" s="12" t="n"/>
       <c r="D56" s="13" t="n"/>
       <c r="E56" s="12" t="n"/>
@@ -1243,7 +1297,7 @@
       <c r="A57" s="6" t="n">
         <v>53</v>
       </c>
-      <c r="B57" s="7" t="n"/>
+      <c r="B57" s="16" t="n"/>
       <c r="C57" s="8" t="n"/>
       <c r="D57" s="9" t="n"/>
       <c r="E57" s="8" t="n"/>
@@ -1255,7 +1309,7 @@
       <c r="A58" s="10" t="n">
         <v>54</v>
       </c>
-      <c r="B58" s="11" t="n"/>
+      <c r="B58" s="17" t="n"/>
       <c r="C58" s="12" t="n"/>
       <c r="D58" s="13" t="n"/>
       <c r="E58" s="12" t="n"/>
@@ -1267,7 +1321,7 @@
       <c r="A59" s="6" t="n">
         <v>55</v>
       </c>
-      <c r="B59" s="7" t="n"/>
+      <c r="B59" s="16" t="n"/>
       <c r="C59" s="8" t="n"/>
       <c r="D59" s="9" t="n"/>
       <c r="E59" s="8" t="n"/>
@@ -1279,7 +1333,7 @@
       <c r="A60" s="10" t="n">
         <v>56</v>
       </c>
-      <c r="B60" s="11" t="n"/>
+      <c r="B60" s="17" t="n"/>
       <c r="C60" s="12" t="n"/>
       <c r="D60" s="13" t="n"/>
       <c r="E60" s="12" t="n"/>
@@ -1291,7 +1345,7 @@
       <c r="A61" s="6" t="n">
         <v>57</v>
       </c>
-      <c r="B61" s="7" t="n"/>
+      <c r="B61" s="16" t="n"/>
       <c r="C61" s="8" t="n"/>
       <c r="D61" s="9" t="n"/>
       <c r="E61" s="8" t="n"/>
@@ -1303,7 +1357,7 @@
       <c r="A62" s="10" t="n">
         <v>58</v>
       </c>
-      <c r="B62" s="11" t="n"/>
+      <c r="B62" s="17" t="n"/>
       <c r="C62" s="12" t="n"/>
       <c r="D62" s="13" t="n"/>
       <c r="E62" s="12" t="n"/>
@@ -1315,7 +1369,7 @@
       <c r="A63" s="6" t="n">
         <v>59</v>
       </c>
-      <c r="B63" s="7" t="n"/>
+      <c r="B63" s="16" t="n"/>
       <c r="C63" s="8" t="n"/>
       <c r="D63" s="9" t="n"/>
       <c r="E63" s="8" t="n"/>
@@ -1327,7 +1381,7 @@
       <c r="A64" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="B64" s="11" t="n"/>
+      <c r="B64" s="17" t="n"/>
       <c r="C64" s="12" t="n"/>
       <c r="D64" s="13" t="n"/>
       <c r="E64" s="12" t="n"/>
@@ -1339,7 +1393,7 @@
       <c r="A65" s="6" t="n">
         <v>61</v>
       </c>
-      <c r="B65" s="7" t="n"/>
+      <c r="B65" s="16" t="n"/>
       <c r="C65" s="8" t="n"/>
       <c r="D65" s="9" t="n"/>
       <c r="E65" s="8" t="n"/>
@@ -1351,7 +1405,7 @@
       <c r="A66" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="B66" s="11" t="n"/>
+      <c r="B66" s="17" t="n"/>
       <c r="C66" s="12" t="n"/>
       <c r="D66" s="13" t="n"/>
       <c r="E66" s="12" t="n"/>
@@ -1363,7 +1417,7 @@
       <c r="A67" s="6" t="n">
         <v>63</v>
       </c>
-      <c r="B67" s="7" t="n"/>
+      <c r="B67" s="16" t="n"/>
       <c r="C67" s="8" t="n"/>
       <c r="D67" s="9" t="n"/>
       <c r="E67" s="8" t="n"/>
@@ -1375,7 +1429,7 @@
       <c r="A68" s="10" t="n">
         <v>64</v>
       </c>
-      <c r="B68" s="11" t="n"/>
+      <c r="B68" s="17" t="n"/>
       <c r="C68" s="12" t="n"/>
       <c r="D68" s="13" t="n"/>
       <c r="E68" s="12" t="n"/>
@@ -1387,7 +1441,7 @@
       <c r="A69" s="6" t="n">
         <v>65</v>
       </c>
-      <c r="B69" s="7" t="n"/>
+      <c r="B69" s="16" t="n"/>
       <c r="C69" s="8" t="n"/>
       <c r="D69" s="9" t="n"/>
       <c r="E69" s="8" t="n"/>
@@ -1399,7 +1453,7 @@
       <c r="A70" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="B70" s="11" t="n"/>
+      <c r="B70" s="17" t="n"/>
       <c r="C70" s="12" t="n"/>
       <c r="D70" s="13" t="n"/>
       <c r="E70" s="12" t="n"/>
@@ -1411,7 +1465,7 @@
       <c r="A71" s="6" t="n">
         <v>67</v>
       </c>
-      <c r="B71" s="7" t="n"/>
+      <c r="B71" s="16" t="n"/>
       <c r="C71" s="8" t="n"/>
       <c r="D71" s="9" t="n"/>
       <c r="E71" s="8" t="n"/>
@@ -1423,7 +1477,7 @@
       <c r="A72" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="B72" s="11" t="n"/>
+      <c r="B72" s="17" t="n"/>
       <c r="C72" s="12" t="n"/>
       <c r="D72" s="13" t="n"/>
       <c r="E72" s="12" t="n"/>
@@ -1435,7 +1489,7 @@
       <c r="A73" s="6" t="n">
         <v>69</v>
       </c>
-      <c r="B73" s="7" t="n"/>
+      <c r="B73" s="16" t="n"/>
       <c r="C73" s="8" t="n"/>
       <c r="D73" s="9" t="n"/>
       <c r="E73" s="8" t="n"/>
@@ -1447,7 +1501,7 @@
       <c r="A74" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="B74" s="11" t="n"/>
+      <c r="B74" s="17" t="n"/>
       <c r="C74" s="12" t="n"/>
       <c r="D74" s="13" t="n"/>
       <c r="E74" s="12" t="n"/>
@@ -1459,7 +1513,7 @@
       <c r="A75" s="6" t="n">
         <v>71</v>
       </c>
-      <c r="B75" s="7" t="n"/>
+      <c r="B75" s="16" t="n"/>
       <c r="C75" s="8" t="n"/>
       <c r="D75" s="9" t="n"/>
       <c r="E75" s="8" t="n"/>
@@ -1471,7 +1525,7 @@
       <c r="A76" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="B76" s="11" t="n"/>
+      <c r="B76" s="17" t="n"/>
       <c r="C76" s="12" t="n"/>
       <c r="D76" s="13" t="n"/>
       <c r="E76" s="12" t="n"/>
@@ -1483,7 +1537,7 @@
       <c r="A77" s="6" t="n">
         <v>73</v>
       </c>
-      <c r="B77" s="7" t="n"/>
+      <c r="B77" s="16" t="n"/>
       <c r="C77" s="8" t="n"/>
       <c r="D77" s="9" t="n"/>
       <c r="E77" s="8" t="n"/>
@@ -1495,7 +1549,7 @@
       <c r="A78" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="B78" s="11" t="n"/>
+      <c r="B78" s="17" t="n"/>
       <c r="C78" s="12" t="n"/>
       <c r="D78" s="13" t="n"/>
       <c r="E78" s="12" t="n"/>
@@ -1507,7 +1561,7 @@
       <c r="A79" s="6" t="n">
         <v>75</v>
       </c>
-      <c r="B79" s="7" t="n"/>
+      <c r="B79" s="16" t="n"/>
       <c r="C79" s="8" t="n"/>
       <c r="D79" s="9" t="n"/>
       <c r="E79" s="8" t="n"/>
@@ -1519,7 +1573,7 @@
       <c r="A80" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="B80" s="11" t="n"/>
+      <c r="B80" s="17" t="n"/>
       <c r="C80" s="12" t="n"/>
       <c r="D80" s="13" t="n"/>
       <c r="E80" s="12" t="n"/>
@@ -1531,7 +1585,7 @@
       <c r="A81" s="6" t="n">
         <v>77</v>
       </c>
-      <c r="B81" s="7" t="n"/>
+      <c r="B81" s="16" t="n"/>
       <c r="C81" s="8" t="n"/>
       <c r="D81" s="9" t="n"/>
       <c r="E81" s="8" t="n"/>
@@ -1543,7 +1597,7 @@
       <c r="A82" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="B82" s="11" t="n"/>
+      <c r="B82" s="17" t="n"/>
       <c r="C82" s="12" t="n"/>
       <c r="D82" s="13" t="n"/>
       <c r="E82" s="12" t="n"/>
@@ -1555,7 +1609,7 @@
       <c r="A83" s="6" t="n">
         <v>79</v>
       </c>
-      <c r="B83" s="7" t="n"/>
+      <c r="B83" s="16" t="n"/>
       <c r="C83" s="8" t="n"/>
       <c r="D83" s="9" t="n"/>
       <c r="E83" s="8" t="n"/>
@@ -1567,7 +1621,7 @@
       <c r="A84" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="B84" s="11" t="n"/>
+      <c r="B84" s="17" t="n"/>
       <c r="C84" s="12" t="n"/>
       <c r="D84" s="13" t="n"/>
       <c r="E84" s="12" t="n"/>
@@ -1579,7 +1633,7 @@
       <c r="A85" s="6" t="n">
         <v>81</v>
       </c>
-      <c r="B85" s="7" t="n"/>
+      <c r="B85" s="16" t="n"/>
       <c r="C85" s="8" t="n"/>
       <c r="D85" s="9" t="n"/>
       <c r="E85" s="8" t="n"/>
@@ -1591,7 +1645,7 @@
       <c r="A86" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="B86" s="11" t="n"/>
+      <c r="B86" s="17" t="n"/>
       <c r="C86" s="12" t="n"/>
       <c r="D86" s="13" t="n"/>
       <c r="E86" s="12" t="n"/>
@@ -1603,7 +1657,7 @@
       <c r="A87" s="6" t="n">
         <v>83</v>
       </c>
-      <c r="B87" s="7" t="n"/>
+      <c r="B87" s="16" t="n"/>
       <c r="C87" s="8" t="n"/>
       <c r="D87" s="9" t="n"/>
       <c r="E87" s="8" t="n"/>
@@ -1615,7 +1669,7 @@
       <c r="A88" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="B88" s="11" t="n"/>
+      <c r="B88" s="17" t="n"/>
       <c r="C88" s="12" t="n"/>
       <c r="D88" s="13" t="n"/>
       <c r="E88" s="12" t="n"/>
@@ -1627,7 +1681,7 @@
       <c r="A89" s="6" t="n">
         <v>85</v>
       </c>
-      <c r="B89" s="7" t="n"/>
+      <c r="B89" s="16" t="n"/>
       <c r="C89" s="8" t="n"/>
       <c r="D89" s="9" t="n"/>
       <c r="E89" s="8" t="n"/>
@@ -1639,7 +1693,7 @@
       <c r="A90" s="10" t="n">
         <v>86</v>
       </c>
-      <c r="B90" s="11" t="n"/>
+      <c r="B90" s="17" t="n"/>
       <c r="C90" s="12" t="n"/>
       <c r="D90" s="13" t="n"/>
       <c r="E90" s="12" t="n"/>
@@ -1651,7 +1705,7 @@
       <c r="A91" s="6" t="n">
         <v>87</v>
       </c>
-      <c r="B91" s="7" t="n"/>
+      <c r="B91" s="16" t="n"/>
       <c r="C91" s="8" t="n"/>
       <c r="D91" s="9" t="n"/>
       <c r="E91" s="8" t="n"/>
@@ -1663,7 +1717,7 @@
       <c r="A92" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="B92" s="11" t="n"/>
+      <c r="B92" s="17" t="n"/>
       <c r="C92" s="12" t="n"/>
       <c r="D92" s="13" t="n"/>
       <c r="E92" s="12" t="n"/>
@@ -1675,7 +1729,7 @@
       <c r="A93" s="6" t="n">
         <v>89</v>
       </c>
-      <c r="B93" s="7" t="n"/>
+      <c r="B93" s="16" t="n"/>
       <c r="C93" s="8" t="n"/>
       <c r="D93" s="9" t="n"/>
       <c r="E93" s="8" t="n"/>
@@ -1687,7 +1741,7 @@
       <c r="A94" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="B94" s="11" t="n"/>
+      <c r="B94" s="17" t="n"/>
       <c r="C94" s="12" t="n"/>
       <c r="D94" s="13" t="n"/>
       <c r="E94" s="12" t="n"/>
@@ -1699,7 +1753,7 @@
       <c r="A95" s="6" t="n">
         <v>91</v>
       </c>
-      <c r="B95" s="7" t="n"/>
+      <c r="B95" s="16" t="n"/>
       <c r="C95" s="8" t="n"/>
       <c r="D95" s="9" t="n"/>
       <c r="E95" s="8" t="n"/>
@@ -1711,7 +1765,7 @@
       <c r="A96" s="10" t="n">
         <v>92</v>
       </c>
-      <c r="B96" s="11" t="n"/>
+      <c r="B96" s="17" t="n"/>
       <c r="C96" s="12" t="n"/>
       <c r="D96" s="13" t="n"/>
       <c r="E96" s="12" t="n"/>
@@ -1723,7 +1777,7 @@
       <c r="A97" s="6" t="n">
         <v>93</v>
       </c>
-      <c r="B97" s="7" t="n"/>
+      <c r="B97" s="16" t="n"/>
       <c r="C97" s="8" t="n"/>
       <c r="D97" s="9" t="n"/>
       <c r="E97" s="8" t="n"/>
@@ -1735,7 +1789,7 @@
       <c r="A98" s="10" t="n">
         <v>94</v>
       </c>
-      <c r="B98" s="11" t="n"/>
+      <c r="B98" s="17" t="n"/>
       <c r="C98" s="12" t="n"/>
       <c r="D98" s="13" t="n"/>
       <c r="E98" s="12" t="n"/>
@@ -1747,7 +1801,7 @@
       <c r="A99" s="6" t="n">
         <v>95</v>
       </c>
-      <c r="B99" s="7" t="n"/>
+      <c r="B99" s="16" t="n"/>
       <c r="C99" s="8" t="n"/>
       <c r="D99" s="9" t="n"/>
       <c r="E99" s="8" t="n"/>
@@ -1759,7 +1813,7 @@
       <c r="A100" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="B100" s="11" t="n"/>
+      <c r="B100" s="17" t="n"/>
       <c r="C100" s="12" t="n"/>
       <c r="D100" s="13" t="n"/>
       <c r="E100" s="12" t="n"/>
@@ -1771,7 +1825,7 @@
       <c r="A101" s="6" t="n">
         <v>97</v>
       </c>
-      <c r="B101" s="7" t="n"/>
+      <c r="B101" s="16" t="n"/>
       <c r="C101" s="8" t="n"/>
       <c r="D101" s="9" t="n"/>
       <c r="E101" s="8" t="n"/>
@@ -1783,7 +1837,7 @@
       <c r="A102" s="10" t="n">
         <v>98</v>
       </c>
-      <c r="B102" s="11" t="n"/>
+      <c r="B102" s="17" t="n"/>
       <c r="C102" s="12" t="n"/>
       <c r="D102" s="13" t="n"/>
       <c r="E102" s="12" t="n"/>
@@ -1795,7 +1849,7 @@
       <c r="A103" s="6" t="n">
         <v>99</v>
       </c>
-      <c r="B103" s="7" t="n"/>
+      <c r="B103" s="16" t="n"/>
       <c r="C103" s="8" t="n"/>
       <c r="D103" s="9" t="n"/>
       <c r="E103" s="8" t="n"/>
@@ -1807,7 +1861,7 @@
       <c r="A104" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="B104" s="11" t="n"/>
+      <c r="B104" s="17" t="n"/>
       <c r="C104" s="12" t="n"/>
       <c r="D104" s="13" t="n"/>
       <c r="E104" s="12" t="n"/>

</xml_diff>

<commit_message>
Fill school name in visitor log
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013FUkLGmYvKevpCsh9ZXdui
</commit_message>
<xml_diff>
--- a/resources/سجل_الزائرات_للمدرسة.xlsx
+++ b/resources/سجل_الزائرات_للمدرسة.xlsx
@@ -615,7 +615,11 @@
         </is>
       </c>
       <c r="B2" s="14" t="n"/>
-      <c r="C2" s="4" t="n"/>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>ب/٩٦ صفوف عليا+ صعوبات التعلم+ م/٤٥</t>
+        </is>
+      </c>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="14" t="n"/>
       <c r="F2" s="2" t="inlineStr">

</xml_diff>